<commit_message>
Fix UI styling, remove tile explore footer, fix Mongoose models and startup scripts
</commit_message>
<xml_diff>
--- a/server/uploads/book1.xlsx
+++ b/server/uploads/book1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anush\OneDrive\Desktop\projects\HRMS system\server\uploads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/84ae2a03b92389ac/Desktop/projects/HRMS system/server/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5490D53F-7A9B-4E3B-A828-58861BCA5C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{5490D53F-7A9B-4E3B-A828-58861BCA5C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A99B9CE-91F5-42B1-A51B-2E28516A0514}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{DCCC6805-F783-44CF-8F5A-645AFE77ABF3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DCCC6805-F783-44CF-8F5A-645AFE77ABF3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="308">
   <si>
     <t>Emp ID</t>
   </si>
@@ -938,12 +938,6 @@
     <t>Anushka</t>
   </si>
   <si>
-    <t>68666cf8cc22e3579418124d</t>
-  </si>
-  <si>
-    <t>Anu</t>
-  </si>
-  <si>
     <t>Trisha</t>
   </si>
   <si>
@@ -963,6 +957,9 @@
   </si>
   <si>
     <t>6907a4d6f37984871bfd0e75</t>
+  </si>
+  <si>
+    <t>Anushka Dutta</t>
   </si>
 </sst>
 </file>
@@ -1429,7 +1426,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>299</v>
@@ -1464,7 +1461,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>299</v>
@@ -1502,7 +1499,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>299</v>
@@ -1537,7 +1534,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>299</v>
@@ -1572,7 +1569,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>299</v>
@@ -1610,7 +1607,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>299</v>
@@ -1648,10 +1645,10 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
@@ -1683,10 +1680,10 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -1721,10 +1718,10 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C10" t="s">
         <v>31</v>
@@ -1756,10 +1753,10 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C11" t="s">
         <v>40</v>
@@ -1794,10 +1791,10 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C12" t="s">
         <v>49</v>
@@ -1832,10 +1829,10 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C13" t="s">
         <v>58</v>
@@ -1867,10 +1864,10 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -1905,10 +1902,10 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C15" t="s">
         <v>21</v>
@@ -1943,10 +1940,10 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
@@ -1978,10 +1975,10 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C17" t="s">
         <v>40</v>
@@ -2013,10 +2010,10 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
@@ -2048,10 +2045,10 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C19" t="s">
         <v>58</v>
@@ -2086,10 +2083,10 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -2124,10 +2121,10 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C21" t="s">
         <v>21</v>
@@ -2162,10 +2159,10 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C22" t="s">
         <v>31</v>
@@ -2197,10 +2194,10 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C23" t="s">
         <v>40</v>
@@ -2235,10 +2232,10 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C24" t="s">
         <v>49</v>
@@ -2273,10 +2270,10 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C25" t="s">
         <v>58</v>
@@ -2311,7 +2308,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>299</v>
@@ -2349,7 +2346,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>299</v>
@@ -2387,7 +2384,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>299</v>
@@ -2422,7 +2419,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>299</v>
@@ -2457,7 +2454,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>299</v>
@@ -2495,7 +2492,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>299</v>
@@ -2530,10 +2527,10 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -2565,10 +2562,10 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C33" t="s">
         <v>21</v>
@@ -2600,10 +2597,10 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C34" t="s">
         <v>31</v>
@@ -2638,10 +2635,10 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C35" t="s">
         <v>40</v>
@@ -2676,10 +2673,10 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C36" t="s">
         <v>49</v>
@@ -2714,10 +2711,10 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C37" t="s">
         <v>58</v>

</xml_diff>